<commit_message>
Regenerate results after 0006: Table A5 per block, block variation limits (Windows run)
</commit_message>
<xml_diff>
--- a/results/tables/excel/table_A5_weighting_rules.xlsx
+++ b/results/tables/excel/table_A5_weighting_rules.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,7 +507,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>no (synthetic)</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -536,7 +536,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>no (synthetic)</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -550,6 +550,64 @@
       </c>
       <c r="G4" t="n">
         <v>4.770701892730803</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>demand_normalized</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>w_f = 1 / D_f, D_f the seasonal demand (rule (v) of Section 2.6); computed from the published demands</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>derived from the published demands</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>0.8499999999996504</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.8499999999996466</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9029454243031589</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5.425915102597673</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>synthetic_single_block_priority</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SYNTHETIC w = 100 for the block least served under uniform weights, 1 for all others; a deliberately one-sided weighting used to show what a contested choice can and cannot do</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>no (synthetic)</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>0.8499999999996504</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.8499999999996504</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.8963109569898047</v>
+      </c>
+      <c r="G6" t="n">
+        <v>4.509109571032459</v>
       </c>
     </row>
   </sheetData>

</xml_diff>